<commit_message>
commit student import template modified
</commit_message>
<xml_diff>
--- a/public/templates/student_import_template.xlsx
+++ b/public/templates/student_import_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Document\WORKING\lavarel_qlgx\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7152F730-370D-4FFD-924A-3D0360245C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF96A41-1FD8-4169-8AA1-FAD759C1E5B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
   <si>
     <t>Tên thánh</t>
   </si>
@@ -178,50 +178,12 @@
   <si>
     <t>DANH SÁCH GHI DANH HỌC SINH</t>
   </si>
-  <si>
-    <r>
-      <t>(*) Nhập dữ liệu từ dòng 6. Không xóa dòng 4 và 5. ten_thanh và giao_ho phải khớp tên trong hệ thống. Hãy đọc hướng dẫn kỹ hơn ở Sheet</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Hướng dẫn</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>NHỚ XÓA DÒNG NÀY NHA!!!</t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -266,37 +228,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF888888"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -445,7 +376,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -457,10 +388,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
@@ -492,32 +423,24 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -828,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L1000"/>
+  <dimension ref="A1:L999"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="7" customWidth="1"/>
@@ -1109,21 +1032,19 @@
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
     </row>
-    <row r="16" spans="1:12" ht="16.05" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
+    <row r="16" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
     </row>
     <row r="17" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="8"/>
@@ -14887,30 +14808,15 @@
       <c r="K999" s="8"/>
       <c r="L999" s="8"/>
     </row>
-    <row r="1000" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1000" s="8"/>
-      <c r="B1000" s="8"/>
-      <c r="C1000" s="8"/>
-      <c r="D1000" s="9"/>
-      <c r="E1000" s="8"/>
-      <c r="F1000" s="8"/>
-      <c r="G1000" s="8"/>
-      <c r="H1000" s="8"/>
-      <c r="I1000" s="9"/>
-      <c r="J1000" s="8"/>
-      <c r="K1000" s="8"/>
-      <c r="L1000" s="8"/>
-    </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
-  <mergeCells count="4">
+  <sheetProtection selectLockedCells="1"/>
+  <mergeCells count="3">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A16:L16"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E15 E17:E1000" xr:uid="{45C970E0-4C01-4AFA-8896-60FCC444E033}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E15 E16:E999" xr:uid="{45C970E0-4C01-4AFA-8896-60FCC444E033}">
       <formula1>"Nam, Nữ"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14931,10 +14837,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="24"/>
+      <c r="C1" s="22"/>
     </row>
     <row r="2" spans="2:3" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2"/>
@@ -14989,10 +14895,10 @@
       <c r="B9" s="2"/>
     </row>
     <row r="10" spans="2:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="25"/>
+      <c r="C10" s="23"/>
     </row>
     <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">

</xml_diff>

<commit_message>
commit student import template modified 2
</commit_message>
<xml_diff>
--- a/public/templates/student_import_template.xlsx
+++ b/public/templates/student_import_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Document\WORKING\lavarel_qlgx\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF96A41-1FD8-4169-8AA1-FAD759C1E5B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91DD1FCE-D98D-4006-AC52-F68431FE2AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14809,7 +14809,7 @@
       <c r="L999" s="8"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection sheet="1" selectLockedCells="1"/>
   <mergeCells count="3">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>